<commit_message>
update(db): update databases on remote repository
</commit_message>
<xml_diff>
--- a/descontos_seguranca/data/auxiliary/aux_gestores.xlsx
+++ b/descontos_seguranca/data/auxiliary/aux_gestores.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sipel\Documents\pipelines-dados-SIPEL\pipelines-dados-SIPEL\descontos_segurança\data\auxiliary\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorg2135259-my.sharepoint.com/personal/controledesempenho_sipel_com_br/Documents/pipelines-dados-SIPEL/descontos_seguranca/data/auxiliary/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F50A09DF-E4B0-4FE7-93BE-6C3F157CCF7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{F50A09DF-E4B0-4FE7-93BE-6C3F157CCF7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{806F32EF-58E3-4D0E-8DE5-C14DDA7E04A4}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="145">
   <si>
     <t>INSPETORES</t>
   </si>
@@ -443,17 +443,39 @@
   </si>
   <si>
     <t>CARLOS NUNES</t>
+  </si>
+  <si>
+    <t>PABLO BRITO - 000000000</t>
+  </si>
+  <si>
+    <t>Frota</t>
+  </si>
+  <si>
+    <t>PABLO BRITO</t>
+  </si>
+  <si>
+    <t>RUBEM FREITAS - 000000000</t>
+  </si>
+  <si>
+    <t>RUBEM FREITAS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -601,16 +623,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -619,8 +642,8 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2069,8 +2092,46 @@
         <v>128</v>
       </c>
     </row>
-    <row r="62" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="63" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="62" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>140</v>
+      </c>
+      <c r="B62" s="22" t="s">
+        <v>141</v>
+      </c>
+      <c r="C62" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="D62" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="E62" s="22" t="s">
+        <v>142</v>
+      </c>
+      <c r="F62" s="22" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>143</v>
+      </c>
+      <c r="B63" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C63" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="D63" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="E63" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="F63" s="22" t="s">
+        <v>129</v>
+      </c>
+    </row>
     <row r="64" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="65" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="66" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>